<commit_message>
Updated FRA_grids_kan25 model - 2026-07-29 13:05
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_kan25/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_kan25/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4E8C82D-26C0-46D7-912A-B0860B746487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{32387859-0507-417F-889E-AB26B8730BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26746,7 +26746,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8386D5D-355A-4310-82A9-E1E734B8608C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A56464AC-8DDC-4ABB-859F-E6A141BA3E9D}">
   <dimension ref="B9:H111"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28804,7 +28804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C2562BF-BE00-4890-8BD8-27E41DFFB595}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE97C6AA-B391-4E5A-BA33-AFD91E1E43AD}">
   <dimension ref="B9:L111"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FRA_grids_kan25 model - 2026-07-29 14:10
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_kan25/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_kan25/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32387859-0507-417F-889E-AB26B8730BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{58E2620F-675F-41BC-A14C-98D41FE19023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26746,7 +26746,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A56464AC-8DDC-4ABB-859F-E6A141BA3E9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BDBA24E-B9E0-45EA-9FF9-ECCEE8210C3B}">
   <dimension ref="B9:H111"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28804,7 +28804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE97C6AA-B391-4E5A-BA33-AFD91E1E43AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3751630E-0234-44B6-8824-7D180CCF52B1}">
   <dimension ref="B9:L111"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>